<commit_message>
feat(streaming-portal): remove Sheet 1 overlapping streams from Sheet 2 in Google Sheet
</commit_message>
<xml_diff>
--- a/05_STREAMING_PORTAL/Google_Sheet_Complete_Cleaned.xlsx
+++ b/05_STREAMING_PORTAL/Google_Sheet_Complete_Cleaned.xlsx
@@ -2654,7 +2654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E130"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2721,12 +2721,12 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Aaryaa Tv</t>
+          <t>Chithiram Tv</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://stream.ottlive.co.in/aryatvtamil/index.m3u8</t>
+          <t>https://cdn-6.pishow.tv/live/1243/master.m3u8</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -2739,21 +2739,21 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Chithiram Tv</t>
+          <t>DD Tamil</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-6.pishow.tv/live/1243/master.m3u8</t>
+          <t>https://cdn-2.pishow.tv/live/26/master.m3u8</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -2775,17 +2775,17 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>DD Tamil</t>
+          <t>Go USA</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-2.pishow.tv/live/26/master.m3u8</t>
+          <t>https://brandusa-gousa-1-in.samsung.wurl.tv/playlist.m3u8</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2802,17 +2802,17 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Fail Army</t>
+          <t>IBC Tamil</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://failarmy-international-in.samsung.wurl.tv/playlist.m3u8</t>
+          <t>https://ibc.massstream.net/IBC/index.m3u8</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2829,17 +2829,17 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Go USA</t>
+          <t>Malai Murasu Tv</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://brandusa-gousa-1-in.samsung.wurl.tv/playlist.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1606/master.m3u8</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2856,12 +2856,12 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>IBC Tamil</t>
+          <t>Malar Tv</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://ibc.massstream.net/IBC/index.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/473/master.m3u8</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -2874,26 +2874,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Isaiaruvi Tv</t>
+          <t>Manorama Tv</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>https://segment.yuppcdn.net/140622/isaiaruvi/playlist.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1479/master.m3u8</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -2901,21 +2901,21 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Kalaignar Tv</t>
+          <t>Mk Six Tv</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>https://segment.yuppcdn.net/240122/kalaignartv/playlist.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1253/master.m3u8</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -2928,21 +2928,21 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Malai Murasu Tv</t>
+          <t>Moon Tv</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/1606/master.m3u8</t>
+          <t>https://player.mslivestream.net/mslive/e10bb900976df9177b9a080314f26f86.sdp/index.m3u8</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2964,12 +2964,12 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Malar Tv</t>
+          <t>News 7 Tv</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/473/master.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1498/master.m3u8</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -2991,17 +2991,17 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Manorama Tv</t>
+          <t>News J Tv</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/1479/master.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1279/master.m3u8</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -3018,12 +3018,12 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Mk Six Tv</t>
+          <t>News tamil Tv</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/1253/master.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1433/master.m3u8</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -3045,12 +3045,12 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>MN Tv</t>
+          <t>Peppers Tv</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>https://mntv.livebox.co.in/mntvhls/live.m3u8</t>
+          <t>https://cdn-2.pishow.tv/live/1383/master.m3u8</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -3063,21 +3063,21 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Moon Tv</t>
+          <t>Polimer news</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>https://player.mslivestream.net/mslive/e10bb900976df9177b9a080314f26f86.sdp/index.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1245/master.m3u8</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -3099,17 +3099,17 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Movie Club 2 Tv</t>
+          <t>Polimer news</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>https://d3gnyty2vddhsg.cloudfront.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/pb-ytipwjqub3kf8/TMC2_IN.m3u8?ads.ads_cdn=cf&amp;ads.cdn=cf</t>
+          <t>https://live-cf-polimernews.dailyhunt.in/master.m3u8</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -3117,26 +3117,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Movie Club Tv</t>
+          <t>Puthiyathalaimurai tv</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>https://sis-global.prod.samsungtv.plus/v1/tvpprd/sc-mp2ar4ca425xo.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1261/master.m3u8</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -3144,26 +3144,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Murasu Tv</t>
+          <t>Rakuten Action Movies</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>https://segment.yuppcdn.net/050522/murasu/playlist.m3u8</t>
+          <t>https://54045f0c40fd442c8b06df076aaf1e85.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-6065/master.m3u8</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -3180,17 +3180,17 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>News 7 Tv</t>
+          <t>Rakuten Family Movies</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/1498/master.m3u8</t>
+          <t>https://e3207568b726401995c25670faaf32e4.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-6203/master.m3u8</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -3198,26 +3198,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>News 7 Tv</t>
+          <t>Rakuten Top Movies</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>https://segment.yuppcdn.net/240122/news7/playlist.m3u8</t>
+          <t>https://0145451975a64b35866170fd2e8fa486.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-5987/master.m3u8</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -3234,17 +3234,17 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>News J Tv</t>
+          <t>Shemaroo Tv</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/1279/master.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/230/master.m3u8</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -3261,17 +3261,17 @@
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>News tamil Tv</t>
+          <t>Sony MAX 2</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/1433/master.m3u8</t>
+          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20MAX%202.m3u8</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -3279,26 +3279,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Peppers Tv</t>
+          <t>Sony MAX HD</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-2.pishow.tv/live/1383/master.m3u8</t>
+          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20MAX%20HD.m3u8</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -3306,26 +3306,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Polimer news</t>
+          <t>Sony PIX HD</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/1245/master.m3u8</t>
+          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20PIX%20HD.m3u8</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -3333,26 +3333,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Polimer news</t>
+          <t>Sony WAH</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>https://live-cf-polimernews.dailyhunt.in/master.m3u8</t>
+          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20WAH.m3u8</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -3360,21 +3360,21 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Puthiyathalaimurai tv</t>
+          <t>Star Vijay HD</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/1261/master.m3u8</t>
+          <t>https://peaky.techcoder40.workers.dev/776.m3u8</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -3387,26 +3387,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Rakuten Action Movies</t>
+          <t>Studio One Tv</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>https://54045f0c40fd442c8b06df076aaf1e85.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-6065/master.m3u8</t>
+          <t>https://cdn-1.pishow.tv/live/276/master.m3u8</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -3414,26 +3414,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Rakuten Family Movies</t>
+          <t>Suriya Tv</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>https://e3207568b726401995c25670faaf32e4.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-6203/master.m3u8</t>
+          <t>https://stream.ottlive.co.in/suryatvtamil/index.m3u8</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -3450,17 +3450,17 @@
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Rakuten Top Movies</t>
+          <t>Suriyan Tv</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>https://0145451975a64b35866170fd2e8fa486.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-5987/master.m3u8</t>
+          <t>https://stream.sscloud7.com/live/suriyantv/index.m3u8</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -3477,12 +3477,12 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Roja HD Tv</t>
+          <t>Thanthi Tv</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>https://live.rojatv.cloud/rojatv/rojatv/index.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1612/master.m3u8</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -3495,26 +3495,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Roja Tv</t>
+          <t>Travel XP HD Tv</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>https://stream.rojatv.cloud/rojatv/rojatv/index.m3u8</t>
+          <t>https://deltatesttatasky.akamaized.net/out/i/968284.m3u8</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -3531,12 +3531,12 @@
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Sanaa Tv</t>
+          <t>Velicham Tv</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>https://vglivessai.akamaized.net/us/v1/master/611d79b11b77e2f571934fd80ca1413453772ac7/b6d9e864-ec16-410a-804d-ccf8f720bfaa/index.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/461/master.m3u8</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -3549,26 +3549,26 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Shemaroo Tv</t>
+          <t>Vendar Tv</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/230/master.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1271/master.m3u8</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -3585,17 +3585,17 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Sirippoli HD</t>
+          <t>We Tv</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>https://yuppmedtaorire.akamaized.net/v1/manifest/a0d007312bfd99c47f76b77ae26b1ccdaae76cb1/siripoli_nim_https/c4e6500f-ea05-4226-810e-2833ee0075ff/0.m3u8</t>
+          <t>https://cdn-3.pishow.tv/live/1530/master.m3u8</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -3603,21 +3603,21 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Sirippoli Tv</t>
+          <t>Win Tv</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>https://segment.yuppcdn.net/240122/siripoli/playlist.m3u8</t>
+          <t>https://cdn-4.pishow.tv/live/1531/master.m3u8</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -3630,31 +3630,31 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Sony MAX 2</t>
+          <t>Chithiram Tv</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20MAX%202.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1243/master.m3u8</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>👶</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -3666,17 +3666,17 @@
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Sony MAX HD</t>
+          <t>DD Tamil</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20MAX%20HD.m3u8</t>
+          <t>https://d2lk5u59tns74c.cloudfront.net/out/v1/abf46b148419409d8469d7a9b0c26563/index.m3u8</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -3684,31 +3684,31 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Sony PIX HD</t>
+          <t>Angel TV</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20PIX%20HD.m3u8</t>
+          <t>https://janya-digimix.akamaized.net/vglive-sk-394914/india/ngrp:angelindia_all/playlist.m3u8</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>🪷</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -3720,22 +3720,22 @@
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Sony WAH</t>
+          <t>Angel TV America</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20WAH.m3u8</t>
+          <t>https://janya-digimix.akamaized.net/vglive-sk-374850/america/ngrp:angelamerica_all/playlist.m3u8</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>🪷</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -3747,22 +3747,22 @@
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>South Station Tv</t>
+          <t>Angel TV Indonesia</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>https://cc-yw7ztecy8do3q.akamaized.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/cc-yw7ztecy8do3q/SS_IN.m3u8</t>
+          <t>https://janya-digimix.akamaized.net/vglive-sk-234616/indonesia/ngrp:angelindonesia_all/playlist.m3u8</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>🪷</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -3774,12 +3774,12 @@
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Star Vijay HD</t>
+          <t>MTA6 Asia</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>https://peaky.techcoder40.workers.dev/776.m3u8</t>
+          <t>https://livemtaasia.akamaized.net/hls/live/2039224/mta6asia/playlist.m3u8</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>🪷</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -3801,39 +3801,39 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Studio One Tv</t>
+          <t>MTA7 Asia</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-1.pishow.tv/live/276/master.m3u8</t>
+          <t>https://livemtaasia.akamaized.net/hls/live/2039224/mtaasia2/playlist.m3u8</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
+          <t>🪷</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Subin Tv</t>
+          <t>National Geographic</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>https://stream.galaxyott.live/live/subintv/index.m3u8</t>
+          <t>http://main.light-ott.net:80/play/live.php?mac=00:1A:79:17:28:41&amp;stream=373017&amp;extension=ts&amp;play_token=zCaGy5dtla</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -3855,12 +3855,12 @@
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Suriya Tv</t>
+          <t>News J</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>https://stream.ottlive.co.in/suryatvtamil/index.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1279/master.m3u8</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>📰</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -3882,12 +3882,12 @@
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Suriyan Tv</t>
+          <t>NTC TV</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>https://stream.sscloud7.com/live/suriyantv/index.m3u8</t>
+          <t>https://galaxyott.live/hls/ntv.m3u8</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -3909,12 +3909,12 @@
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Thalaa Tv</t>
+          <t>Oli TV</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>https://streams2.sofast.tv/ptnr-yupptv/title-THALAA-TV-TAM/sofastplayout/981f8f06-782a-4962-b5e0-7dcccd65279c_0_HLS/manifest.m3u8</t>
+          <t>https://live.olidigital.in/olitv/olitv/index.m3u8</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -3927,21 +3927,21 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Thanthi Tv</t>
+          <t>Raj Musix Tamil</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>https://cdn-3.pishow.tv/live/1612/master.m3u8</t>
+          <t>https://livestream.rajtv.tv/hlslive/Admin/px08241087/live/Raj_Musix/master_1.m3u8</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -3951,24 +3951,24 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
+          <t>🎵</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Tharun Movies</t>
+          <t>Raj TV</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>https://streaming.livebox.co.in/tharunmovieshls/live.m3u8</t>
+          <t>https://livestream.rajtv.tv/hlslive/Admin/px08241087/live/RAJTV/master_1.m3u8</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -3990,17 +3990,17 @@
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Toonami Movie</t>
+          <t>Sooriyan TV</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>http://api.toonamiaftermath.com:3000/movies/playlist.m3u8</t>
+          <t>https://live20.bozztv.com/giatv/giatv-Infinittyott/Infinittyott/playlist.m3u8</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -4017,22 +4017,22 @@
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Travel XP HD Tv</t>
+          <t>Vijay Takkar APAC</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>https://deltatesttatasky.akamaized.net/out/i/968284.m3u8</t>
+          <t>https://tglmp01.akamaized.net/out/v1/c1071012b73f4f189b202e1529e8f802/manifest.mpd</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -4044,12 +4044,12 @@
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>TVI HD</t>
+          <t>YET TV</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>https://live.cmr24.fm/TVI/HD/chunks.m3u8</t>
+          <t>https://live.yettelevision.com:5443/LiveApp/streams/yettv.m3u8</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -4062,21 +4062,21 @@
           <t>📺</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Dead</t>
         </is>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Ultimate HD Tv</t>
+          <t>Zee Tamil News</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>https://stream.ottlive.co.in/utvtamil/index.m3u8</t>
+          <t>https://raw.githubusercontent.com/amazeyourself/adaptive-streams/refs/heads/main/streams/in/ZMCL/ZeeTamilNews.m3u8</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -4086,2089 +4086,10 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>📰</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Ultimate Tv</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>https://mumbai-edge.smartplaytv.in/utv/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Vaanavil Tv</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>https://6n3yope4d9ok-hls-live.5centscdn.com/vaanavil/TV.stream/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Velicham Tv</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>https://cdn-3.pishow.tv/live/461/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>Vendar Tv</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>https://cdn-3.pishow.tv/live/1271/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>We Tv</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>https://cdn-3.pishow.tv/live/1530/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>Malayalam</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Win Tv</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>https://cdn-4.pishow.tv/live/1531/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E59" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Zee South Flix Tv</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>https://amg00862-amg00862c9-amgplt0173.playout.now3.amagi.tv/playlist/amg00862-amg00862c9-amgplt0173/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>Hindi</t>
-        </is>
-      </c>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>7s Music Tv</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>https://cdn.pishow.tv/ott/live/1257/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>🎵</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Chithiram Tv</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>https://cdn.pishow.tv/ott/live/1243/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>👶</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>DD Tamil</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>https://d2lk5u59tns74c.cloudfront.net/out/v1/abf46b148419409d8469d7a9b0c26563/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>Thanthi Tv</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>https://streams.tangotv.in/THANTHITV/ORIGIN/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>📰</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>Velicham Tv</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt05.tangotv.in/87NeALx2VALICHAMPLUS/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>☀️</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>Win Tv</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt06.tangotv.in/qYyB8fXVWINTV/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>Aaseervatham TV</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt04.tangotv.in/m18aqlK4AASEERVATHAMTV/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="20" customHeight="1">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Aastha Tamil</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>https://aasthaott.akamaized.net/110923/smil:aasthatamil.smil/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>Angel TV</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>https://janya-digimix.akamaized.net/vglive-sk-394914/india/ngrp:angelindia_all/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Angel TV America</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>https://janya-digimix.akamaized.net/vglive-sk-374850/america/ngrp:angelamerica_all/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>Angel TV Indo-China</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>https://janya-digimix.akamaized.net/vglive-sk-703035/indochina/ngrp:angelindochina_all/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>Angel TV Indonesia</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>https://janya-digimix.akamaized.net/vglive-sk-234616/indonesia/ngrp:angelindonesia_all/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>Arputhar Yesu TV</t>
-        </is>
-      </c>
-      <c r="B73" s="3" t="inlineStr">
-        <is>
-          <t>https://account33.livebox.co.in/jesushelpshls/live.m3u8</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>Colors Tamil HD</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>https://da86m1sqpm3o0.cloudfront.net/28072023/smil:colorstamilhd11.smil/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>✨</t>
-        </is>
-      </c>
-      <c r="E74" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>Dharsan TV</t>
-        </is>
-      </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>https://cable91tataplay.akamaized.net/live/dharshantv/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E75" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>ETV Bal Bharat</t>
-        </is>
-      </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>http://103.185.24.134:3001/ETV-BAL-BHARAT/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>👶</t>
-        </is>
-      </c>
-      <c r="E76" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="20" customHeight="1">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>Hebron TV</t>
-        </is>
-      </c>
-      <c r="B77" s="3" t="inlineStr">
-        <is>
-          <t>https://account20.livebox.co.in/charleshls/live.m3u8</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>Hosanna TV</t>
-        </is>
-      </c>
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>https://asia.mslivestream.net/mslive/bfba54c5c96a6359e2da0ca35f4998af.sdp/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D78" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="20" customHeight="1">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>Hungama TV</t>
-        </is>
-      </c>
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>http://103.185.24.134:3001/HUNGAMA/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>👶</t>
-        </is>
-      </c>
-      <c r="E79" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="20" customHeight="1">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>Joy TV</t>
-        </is>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>https://ktismaservers.in:3412/live/joytvlive.m3u8</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D80" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="20" customHeight="1">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>Kalaignar Murasu</t>
-        </is>
-      </c>
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>https://yuppmedtaorire.akamaized.net/v1/master/a0d007312bfd99c47f76b77ae26b1ccdaae76cb1/murasu_nim_https/050522/murasu/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D81" s="4" t="inlineStr">
-        <is>
-          <t>📰</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="20" customHeight="1">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>Life TV</t>
-        </is>
-      </c>
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>https://lifetv.livebox.co.in/lifetvhls/lifetv.m3u8</t>
-        </is>
-      </c>
-      <c r="C82" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D82" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="20" customHeight="1">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>Madha TV</t>
-        </is>
-      </c>
-      <c r="B83" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt07.tangotv.in/zHjX9OFlMADHATV/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="20" customHeight="1">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>Madhimugam TV</t>
-        </is>
-      </c>
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt01.tangotv.in/O5aw8Zn3MATHIMUGAMTV/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D84" s="4" t="inlineStr">
-        <is>
-          <t>📰</t>
-        </is>
-      </c>
-      <c r="E84" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="20" customHeight="1">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>Makkal TV (576i)</t>
-        </is>
-      </c>
-      <c r="B85" s="3" t="inlineStr">
-        <is>
-          <t>https://5k8q87azdy4v-hls-live.wmncdn.net/MAKKAL/271ddf829afeece44d8732757fba1a66.sdp/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E85" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="20" customHeight="1">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>Mei Alai TV</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t>https://meialai.iptelevishion.com/meialai/2/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C86" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E86" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="20" customHeight="1">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>MK Six</t>
-        </is>
-      </c>
-      <c r="B87" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt06.tangotv.in/qYyB8fXVMKSIX/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C87" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D87" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E87" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="20" customHeight="1">
-      <c r="A88" s="2" t="inlineStr">
-        <is>
-          <t>MTA6 Asia</t>
-        </is>
-      </c>
-      <c r="B88" s="3" t="inlineStr">
-        <is>
-          <t>https://livemtaasia.akamaized.net/hls/live/2039224/mta6asia/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C88" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D88" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="20" customHeight="1">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <t>MTA7 Asia</t>
-        </is>
-      </c>
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t>https://livemtaasia.akamaized.net/hls/live/2039224/mtaasia2/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C89" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D89" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E89" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="20" customHeight="1">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>National Geographic</t>
-        </is>
-      </c>
-      <c r="B90" s="3" t="inlineStr">
-        <is>
-          <t>http://main.light-ott.net:80/play/live.php?mac=00:1A:79:17:28:41&amp;stream=373017&amp;extension=ts&amp;play_token=zCaGy5dtla</t>
-        </is>
-      </c>
-      <c r="C90" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="20" customHeight="1">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>NDTV Good Times</t>
-        </is>
-      </c>
-      <c r="B91" s="3" t="inlineStr">
-        <is>
-          <t>https://amg01448-samsungin-ndtvgoodtimes-samsungin-ad-gp.amagi.tv/playlist/amg01448-samsungin-ndtvgoodtimes-samsungin/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C91" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E91" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>News18 Tamil Nadu</t>
-        </is>
-      </c>
-      <c r="B92" s="3" t="inlineStr">
-        <is>
-          <t>https://n18syndication.akamaized.net/bpk-tv/News18_Tamil_Nadu_NW18_MOB/output01/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C92" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>📰</t>
-        </is>
-      </c>
-      <c r="E92" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="20" customHeight="1">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>News J</t>
-        </is>
-      </c>
-      <c r="B93" s="3" t="inlineStr">
-        <is>
-          <t>https://cdn.pishow.tv/ott/live/1279/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>📰</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="20" customHeight="1">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>News Tamil 24x7</t>
-        </is>
-      </c>
-      <c r="B94" s="3" t="inlineStr">
-        <is>
-          <t>https://cdn.pishow.tv/ott/live/1433/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C94" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D94" s="4" t="inlineStr">
-        <is>
-          <t>📰</t>
-        </is>
-      </c>
-      <c r="E94" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="20" customHeight="1">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>NH Tamil Gold</t>
-        </is>
-      </c>
-      <c r="B95" s="3" t="inlineStr">
-        <is>
-          <t>https://d3arbp6l7f096k.cloudfront.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/pb-gv6wgpbb4mgwk/playlist.m3u8?ads.ads_cdn=cf&amp;ads.app_domain=APP_DOMAIN&amp;ads.cdn=cf</t>
-        </is>
-      </c>
-      <c r="C95" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>🎬</t>
-        </is>
-      </c>
-      <c r="E95" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="20" customHeight="1">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>Nickelodeon</t>
-        </is>
-      </c>
-      <c r="B96" s="3" t="inlineStr">
-        <is>
-          <t>http://103.185.24.134:3001/NICK/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C96" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>👶</t>
-        </is>
-      </c>
-      <c r="E96" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="20" customHeight="1">
-      <c r="A97" s="2" t="inlineStr">
-        <is>
-          <t>NTC TV</t>
-        </is>
-      </c>
-      <c r="B97" s="3" t="inlineStr">
-        <is>
-          <t>https://galaxyott.live/hls/ntv.m3u8</t>
-        </is>
-      </c>
-      <c r="C97" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D97" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E97" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="20" customHeight="1">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>Oli TV</t>
-        </is>
-      </c>
-      <c r="B98" s="3" t="inlineStr">
-        <is>
-          <t>https://live.olidigital.in/olitv/olitv/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C98" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D98" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E98" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="20" customHeight="1">
-      <c r="A99" s="2" t="inlineStr">
-        <is>
-          <t>OM TV</t>
-        </is>
-      </c>
-      <c r="B99" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt01.tangotv.in/O5aw8Zn3OMTV/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C99" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D99" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E99" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="20" customHeight="1">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>Polimer TV</t>
-        </is>
-      </c>
-      <c r="B100" s="3" t="inlineStr">
-        <is>
-          <t>https://cdn.pishow.tv/ott/live/1241/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C100" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D100" s="4" t="inlineStr">
-        <is>
-          <t>📰</t>
-        </is>
-      </c>
-      <c r="E100" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="20" customHeight="1">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>Puthiya Thalaimurai</t>
-        </is>
-      </c>
-      <c r="B101" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt07.tangotv.in/zHjX9OFlPUTHIYAEXPRESS/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C101" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D101" s="4" t="inlineStr">
-        <is>
-          <t>📰</t>
-        </is>
-      </c>
-      <c r="E101" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="20" customHeight="1">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>Puthuyugam TV</t>
-        </is>
-      </c>
-      <c r="B102" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt04.tangotv.in/m18aqlK4PUTHUYUGAMTV/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C102" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D102" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E102" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="20" customHeight="1">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>Raj Digital Plus</t>
-        </is>
-      </c>
-      <c r="B103" s="3" t="inlineStr">
-        <is>
-          <t>https://livestream.rajtv.tv/hlslive/Admin/px08241087/live/RajTV_Digital_plus/master_1.m3u8</t>
-        </is>
-      </c>
-      <c r="C103" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D103" s="4" t="inlineStr">
-        <is>
-          <t>🎬</t>
-        </is>
-      </c>
-      <c r="E103" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="20" customHeight="1">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>Raj Musix Tamil</t>
-        </is>
-      </c>
-      <c r="B104" s="3" t="inlineStr">
-        <is>
-          <t>https://livestream.rajtv.tv/hlslive/Admin/px08241087/live/Raj_Musix/master_1.m3u8</t>
-        </is>
-      </c>
-      <c r="C104" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D104" s="4" t="inlineStr">
-        <is>
-          <t>🎵</t>
-        </is>
-      </c>
-      <c r="E104" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="20" customHeight="1">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>Raj TV</t>
-        </is>
-      </c>
-      <c r="B105" s="3" t="inlineStr">
-        <is>
-          <t>https://livestream.rajtv.tv/hlslive/Admin/px08241087/live/RAJTV/master_1.m3u8</t>
-        </is>
-      </c>
-      <c r="C105" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D105" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E105" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="20" customHeight="1">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>Sai TV</t>
-        </is>
-      </c>
-      <c r="B106" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt03.tangotv.in/Dsly5z3HSAITV/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C106" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D106" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E106" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="20" customHeight="1">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>Sairam TV</t>
-        </is>
-      </c>
-      <c r="B107" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt04.tangotv.in/m18aqlK4SAIRAMTV/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C107" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D107" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E107" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>Sana Plus</t>
-        </is>
-      </c>
-      <c r="B108" s="3" t="inlineStr">
-        <is>
-          <t>https://mumbai-edge.smartplaytv.in/SanaPlusHD/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C108" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D108" s="4" t="inlineStr">
-        <is>
-          <t>🎵</t>
-        </is>
-      </c>
-      <c r="E108" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="20" customHeight="1">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>Sankara TV</t>
-        </is>
-      </c>
-      <c r="B109" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt05.tangotv.in/87NeALx2SRISANKARA/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C109" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D109" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E109" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="20" customHeight="1">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>Sivan TV</t>
-        </is>
-      </c>
-      <c r="B110" s="3" t="inlineStr">
-        <is>
-          <t>http://sivantv.livebox.co.in/sivantvhls/sivan.m3u8</t>
-        </is>
-      </c>
-      <c r="C110" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D110" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E110" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="20" customHeight="1">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>Sonic</t>
-        </is>
-      </c>
-      <c r="B111" s="3" t="inlineStr">
-        <is>
-          <t>http://103.185.24.134:3001/SONIC/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C111" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>👶</t>
-        </is>
-      </c>
-      <c r="E111" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="20" customHeight="1">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>Sony BBC Earth HD</t>
-        </is>
-      </c>
-      <c r="B112" s="3" t="inlineStr">
-        <is>
-          <t>https://cloudplay-sonyliv.pages.dev/bbcearthhd.m3u8</t>
-        </is>
-      </c>
-      <c r="C112" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D112" s="4" t="inlineStr">
-        <is>
-          <t>✨</t>
-        </is>
-      </c>
-      <c r="E112" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>Sony Sports Ten 4</t>
-        </is>
-      </c>
-      <c r="B113" s="3" t="inlineStr">
-        <is>
-          <t>https://cloudplay-sonyliv.pages.dev/ten4.m3u8</t>
-        </is>
-      </c>
-      <c r="C113" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D113" s="4" t="inlineStr">
-        <is>
-          <t>🏏</t>
-        </is>
-      </c>
-      <c r="E113" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>Sony Yay!</t>
-        </is>
-      </c>
-      <c r="B114" s="3" t="inlineStr">
-        <is>
-          <t>https://cloudplay-sonyliv.pages.dev/yay.m3u8</t>
-        </is>
-      </c>
-      <c r="C114" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D114" s="4" t="inlineStr">
-        <is>
-          <t>👶</t>
-        </is>
-      </c>
-      <c r="E114" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="20" customHeight="1">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>Sooriyan TV</t>
-        </is>
-      </c>
-      <c r="B115" s="3" t="inlineStr">
-        <is>
-          <t>https://live20.bozztv.com/giatv/giatv-Infinittyott/Infinittyott/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C115" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D115" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E115" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="20" customHeight="1">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>Star Vijay</t>
-        </is>
-      </c>
-      <c r="B116" s="3" t="inlineStr">
-        <is>
-          <t>https://da86m1sqpm3o0.cloudfront.net/28072023/smil:starvijayuk.smil/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C116" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D116" s="4" t="inlineStr">
-        <is>
-          <t>⭐</t>
-        </is>
-      </c>
-      <c r="E116" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="20" customHeight="1">
-      <c r="A117" s="2" t="inlineStr">
-        <is>
-          <t>Super Hungama</t>
-        </is>
-      </c>
-      <c r="B117" s="3" t="inlineStr">
-        <is>
-          <t>http://103.185.24.134:3001/SUPER-HUNGAMA/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C117" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D117" s="4" t="inlineStr">
-        <is>
-          <t>👶</t>
-        </is>
-      </c>
-      <c r="E117" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="20" customHeight="1">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>SVBC 2</t>
-        </is>
-      </c>
-      <c r="B118" s="3" t="inlineStr">
-        <is>
-          <t>https://player.mslivestream.net/tamil/ac206e74d75b285755ee4924df87d951.sdp/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C118" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D118" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E118" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="20" customHeight="1">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>Tamil Janam</t>
-        </is>
-      </c>
-      <c r="B119" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt01.tangotv.in/O5aw8Zn3JANAMTVTAMIL/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C119" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D119" s="4" t="inlineStr">
-        <is>
-          <t>📰</t>
-        </is>
-      </c>
-      <c r="E119" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="20" customHeight="1">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>Tamilan TV</t>
-        </is>
-      </c>
-      <c r="B120" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt04.tangotv.in/m18aqlK4TAMILANTELEVISION/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C120" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D120" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E120" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="20" customHeight="1">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>Travelxp HD</t>
-        </is>
-      </c>
-      <c r="B121" s="3" t="inlineStr">
-        <is>
-          <t>https://amg00416-amg00416c9-samsung-in-4882.playouts.now.amagi.tv/playlist/amg00416-travelxp-travelxphd-samsungin/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C121" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D121" s="4" t="inlineStr">
-        <is>
-          <t>🌍</t>
-        </is>
-      </c>
-      <c r="E121" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="20" customHeight="1">
-      <c r="A122" s="2" t="inlineStr">
-        <is>
-          <t>Vasanth TV</t>
-        </is>
-      </c>
-      <c r="B122" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt04.tangotv.in/m18aqlK4VASANTHTV/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C122" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D122" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E122" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="20" customHeight="1">
-      <c r="A123" s="2" t="inlineStr">
-        <is>
-          <t>Vendhar TV</t>
-        </is>
-      </c>
-      <c r="B123" s="3" t="inlineStr">
-        <is>
-          <t>https://mumt04.tangotv.in/m18aqlK4VENDHARTV/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C123" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D123" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E123" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="20" customHeight="1">
-      <c r="A124" s="2" t="inlineStr">
-        <is>
-          <t>Vijay Takkar APAC</t>
-        </is>
-      </c>
-      <c r="B124" s="3" t="inlineStr">
-        <is>
-          <t>https://tglmp01.akamaized.net/out/v1/c1071012b73f4f189b202e1529e8f802/manifest.mpd</t>
-        </is>
-      </c>
-      <c r="C124" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D124" s="4" t="inlineStr">
-        <is>
-          <t>🎵</t>
-        </is>
-      </c>
-      <c r="E124" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="20" customHeight="1">
-      <c r="A125" s="2" t="inlineStr">
-        <is>
-          <t>Village TV</t>
-        </is>
-      </c>
-      <c r="B125" s="3" t="inlineStr">
-        <is>
-          <t>https://live.villagetv.net/villagetv/hd/index.m3u8</t>
-        </is>
-      </c>
-      <c r="C125" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D125" s="4" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E125" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="20" customHeight="1">
-      <c r="A126" s="2" t="inlineStr">
-        <is>
-          <t>WOW Kidz Tamil</t>
-        </is>
-      </c>
-      <c r="B126" s="3" t="inlineStr">
-        <is>
-          <t>https://yuppparoriglin.akamaized.net/181224/smil:wowkidztam.smil/playlist.m3u8?hdnts=st=1735898689~exp=1835898688~acl=*~hmac=f5fe24724fe05481e3841f9eb5ab8efdee0a3dd83645ae9dcf45703f525bab7b</t>
-        </is>
-      </c>
-      <c r="C126" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D126" s="4" t="inlineStr">
-        <is>
-          <t>👶</t>
-        </is>
-      </c>
-      <c r="E126" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="20" customHeight="1">
-      <c r="A127" s="2" t="inlineStr">
-        <is>
-          <t>YET Max</t>
-        </is>
-      </c>
-      <c r="B127" s="3" t="inlineStr">
-        <is>
-          <t>https://live.yettelevision.com:5443/LiveApp/streams/yettv2.m3u8</t>
-        </is>
-      </c>
-      <c r="C127" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D127" s="4" t="inlineStr">
-        <is>
-          <t>🎵</t>
-        </is>
-      </c>
-      <c r="E127" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" ht="20" customHeight="1">
-      <c r="A128" s="2" t="inlineStr">
-        <is>
-          <t>YET TV</t>
-        </is>
-      </c>
-      <c r="B128" s="3" t="inlineStr">
-        <is>
-          <t>https://live.yettelevision.com:5443/LiveApp/streams/yettv.m3u8</t>
-        </is>
-      </c>
-      <c r="C128" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D128" s="4" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E128" s="7" t="inlineStr">
-        <is>
-          <t>Dead</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" ht="20" customHeight="1">
-      <c r="A129" s="2" t="inlineStr">
-        <is>
-          <t>Zee Tamil HD</t>
-        </is>
-      </c>
-      <c r="B129" s="3" t="inlineStr">
-        <is>
-          <t>https://da86m1sqpm3o0.cloudfront.net/28072023/smil:zeetamil1.smil/playlist.m3u8</t>
-        </is>
-      </c>
-      <c r="C129" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D129" s="4" t="inlineStr">
-        <is>
-          <t>✨</t>
-        </is>
-      </c>
-      <c r="E129" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" ht="20" customHeight="1">
-      <c r="A130" s="2" t="inlineStr">
-        <is>
-          <t>Zee Tamil News</t>
-        </is>
-      </c>
-      <c r="B130" s="3" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/amazeyourself/adaptive-streams/refs/heads/main/streams/in/ZMCL/ZeeTamilNews.m3u8</t>
-        </is>
-      </c>
-      <c r="C130" s="4" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D130" s="4" t="inlineStr">
-        <is>
-          <t>📰</t>
-        </is>
-      </c>
-      <c r="E130" s="5" t="inlineStr">
         <is>
           <t>Live</t>
         </is>

</xml_diff>